<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.002-04 Les carottes d'Amir
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.002-04.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.002-04.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut des carottes orange pour la soupe. D'abord le jardin : le tuyau est froid, une feuille lisse. Le manteau vert va au crochet. Plus tard le sac cache le crochet. Amir le déplace, reprend le manteau. Au marché les carottes. Deux sorties, le même manteau.</t>
+          <t>La cuillère en bois tient dans un verre. Un éclat de cuillère brille, pâle. La soupe est trop claire. Amir veut des carottes, maintenant. Il court sans le manteau : l'air pique, le sac tombe. Papa s'accroupit. Le manteau vert, le jardin, des fanes trop vertes. Au crochet, le sac cache le manteau. Amir refuse de foncer. L'éclat penche vers le crochet. Il reprend le manteau. Au marché, les carottes. Dans le verre, l'éclat porte une trace orange.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une cuillère en bois sèche près de l'évier. La soupe sent encore dans la cuisine. La vitre a un peu de buée. Dehors, le tuyau d'arrosage est enroulé. Papa plie un sac de toile. Amir, tu as vu la buée ? Oui. On dirait un nuage. En ce moment, Amir essuie un peu la buée. Son manteau vert attend au crochet. On va d'abord au jardin. Le tuyau a peut-être de l'eau. Avant de sortir, on prend le manteau. Amir prend le manteau vert. Il est un peu épais. Amir glisse un bras, puis l'autre. Tu es prêt ? Oui, papa. Papa lace les chaussures d'Amir. Ils vont au jardin. L'air est frais. Amir touche une feuille lisse. Elle sent le jardin. Oui. Un peu l'herbe. Un peu l'eau. Le tuyau d'arrosage est froid. Amir le touche du doigt. Il est froid ! Oui. C'est l'heure de rentrer. Amir entre. Il retire le manteau. Il le raccroche au crochet. Le manteau vert est à sa place. Plus tard, le sac de toile attend. On va au marché, maintenant. Pour les carottes de la soupe. Amir se souvient. Il va vers le crochet. Le sac de toile cache le manteau. Je ne vois plus le manteau. Le sac est devant. Tu peux le déplacer ? Amir pousse le sac tout doux. Le manteau vert réapparaît. Avant de sortir, il le prend. Le même manteau vert. Tu t'es souvenu tout seul. Au marché, ça sent le pain. Papa achète une botte de carottes. Elles sont orange. Oui. On les met dans le sac. Puis ils rentrent. Amir raccroche encore le manteau. Le crochet fait le même petit bruit. Deux fois, papa. Oui. Deux fois. Amir pose le sac de toile. Les carottes font un petit bruit. Tu as fini de poser le sac ? Oui, papa.</t>
+          <t>La cuillère en bois tient dans un verre. Elle sèche, un peu penchée, près de l'évier. Un éclat de cuillère brille sur le bois. Il est pâle, lisse, et il sent la soupe. La casserole fume, trop claire. Il manque l'orange, papa. Les carottes, Amir ? Oui, maintenant ! La buée dessine un trait tordu sur la vitre. Dehors, le tuyau d'arrosage dort enroulé. Papa plie le sac de toile, près du crochet. Amir, tu as vu l'éclat ? Oui, il brille. En ce moment, Amir veut les carottes. On y va, tout de suite ! D'abord le jardin. Une carotte est peut-être prête. Amir saisit le sac de toile. Il court vers la porte, sans le manteau. Je sors, papa ! La porte s'ouvre. L'air froid pique les poignets. La sangle glisse, le sac tombe. Aïe ! Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tes poignets sont froids ? Oui. Le sac est tombé. Le manteau vert attend au crochet. Ce manteau est un peu épais. Le tissu gratte sous les doigts. Amir glisse un bras, puis l'autre. Tu es prêt ? Oui, papa. Ils passent au jardin. Une dalle est froide sous la semelle. Le sol pique. Le coin du tuyau sent l'eau. L'air sent l'herbe mouillée. Amir touche une feuille lisse. Elle sent le jardin. Regarde les fanes. Les fanes sont petites, trop vertes. Je peux tirer ? Elles sont trop petites. Amir lâche la fane. Pas d'orange. Pas cette fois. Le marché a des carottes. Le tuyau d'arrosage est froid sous le doigt. Il est froid ! On rentre. Amir retire le manteau. Il le raccroche au crochet. Le crochet fait un petit tic.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une cuillère en bois sèche près de l'évier. La soupe sent encore dans la cuisine. La vitre a un peu de buée. Dehors, le tuyau d'arrosage est enroulé. Papa plie un sac de toile. Amir, tu as vu la buée ? Oui. On dirait un nuage. En ce moment, Amir essuie un peu la buée. Son manteau vert attend au crochet. On va d'abord au jardin. Le tuyau a peut-être de l'eau. Avant de sortir, on prend le manteau. Amir prend le manteau vert. Il est un peu épais. Amir glisse un bras, puis l'autre. Tu es prêt ? Oui, papa. Papa lace les chaussures d'Amir. Ils vont au jardin. L'air est frais. Amir touche une feuille lisse. Elle sent le jardin. Oui. Un peu l'herbe. Un peu l'eau. Le tuyau d'arrosage est froid. Amir le touche du doigt. Il est froid ! Oui. C'est l'heure de rentrer. Amir entre. Il retire le manteau. Il le raccroche au crochet. Le manteau vert est à sa place. Plus tard, le sac de toile attend. On va au marché, maintenant. Pour les carottes de la soupe. Amir se souvient. Il va vers le crochet. Le sac de toile cache le manteau. Je ne vois plus le manteau. Le sac est devant. Tu peux le déplacer ? Amir pousse le sac tout doux. Le manteau vert réapparaît. Avant de sortir, il le prend. Le même manteau vert. Tu t'es souvenu tout seul. Au marché, ça sent le pain. Papa achète une botte de carottes. Elles sont orange. Oui. On les met dans le sac. Puis ils rentrent. Amir raccroche encore le manteau. Le crochet fait le même petit bruit. Deux fois, papa. Oui. Deux fois. Amir pose le sac de toile. Les carottes font un petit bruit. Tu as fini de poser le sac ? Oui, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La cuillère en bois tient dans un verre. Elle sèche, un peu penchée, près de l'évier. Un &lt;emphasis level="moderate"&gt;éclat de cuillère&lt;/emphasis&gt; brille sur le bois. Il est pâle, lisse, et il sent la soupe. La casserole fume, trop claire. Il manque l'orange, papa. Les carottes, Amir ? Oui, maintenant ! La buée dessine un trait tordu sur la vitre. Dehors, le tuyau d'arrosage dort enroulé. Papa plie le sac de toile, près du crochet. Amir, tu as vu l'éclat ? Oui, il brille. En ce moment, Amir veut les carottes. On y va, tout de suite ! D'abord le jardin. Une carotte est peut-être prête. Amir saisit le sac de toile. Il court vers la porte, sans le manteau. Je sors, papa ! La porte s'ouvre. L'air froid pique les poignets. La sangle glisse, le sac tombe. Aïe ! Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tes poignets sont froids ? Oui. Le sac est tombé. Le manteau vert attend au crochet. Ce manteau est un peu épais. Le tissu gratte sous les doigts. Amir glisse un bras, puis l'autre. Tu es prêt ? Oui, papa. Ils passent au jardin. Une dalle est froide sous la semelle. Le sol pique. Le coin du tuyau sent l'eau. L'air sent l'herbe mouillée. Amir touche une feuille lisse. Elle sent le jardin. Regarde les fanes. Les fanes sont petites, trop vertes. Je peux tirer ? Elles sont trop petites. Amir lâche la fane. Pas d'orange. Pas cette fois. Le marché a des carottes. Le tuyau d'arrosage est froid sous le doigt. Il est froid ! On rentre. Amir retire le manteau. Il le raccroche au crochet. Le crochet fait un petit tic.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Violette est près de la porte. Papa lace ses chaussures. Papa dit : on va au jardin. Avant de sortir, Violette prend son &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Le manteau est vert. Il est un peu épais. Violette glisse un bras, puis l'autre. Ils vont au jardin. L'air est frais. Violette touche une feuille lisse. Papa dit : on rentre. Violette entre. Elle retire le manteau. Elle le raccroche au crochet. Le manteau est à sa place. Plus tard, papa dit : on va au marché. Violette se souvient. Avant de sortir, elle prend le manteau. Au marché, ça sent le pain. Puis ils rentrent. Violette raccroche encore le manteau. Même leçon, autre sortie. Papa dit : merci Violette. [pause]</t>
+          <t>La cuillère en bois tient dans un verre. Elle sèche, un peu penchée, près de l'évier. Un &lt;emphasis&gt;éclat de cuillère&lt;/emphasis&gt; brille sur le bois. Il est pâle, lisse, et il sent la soupe. La casserole fume, trop claire. Il manque l'orange, papa. Les carottes, Amir ? Oui, maintenant ! La buée dessine un trait tordu sur la vitre. Dehors, le tuyau d'arrosage dort enroulé. Papa plie le sac de toile, près du crochet. Amir, tu as vu l'éclat ? Oui, il brille. En ce moment, Amir veut les carottes. On y va, tout de suite ! D'abord le jardin. Une carotte est peut-être prête. Amir saisit le sac de toile. Il court vers la porte, sans le manteau. Je sors, papa ! La porte s'ouvre. L'air froid pique les poignets. La sangle glisse, le sac tombe. Aïe ! Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tes poignets sont froids ? Oui. Le sac est tombé. Le manteau vert attend au crochet. Ce manteau est un peu épais. Le tissu gratte sous les doigts. Amir glisse un bras, puis l'autre. Tu es prêt ? Oui, papa. Ils passent au jardin. Une dalle est froide sous la semelle. Le sol pique. Le coin du tuyau sent l'eau. L'air sent l'herbe mouillée. Amir touche une feuille lisse. Elle sent le jardin. Regarde les fanes. Les fanes sont petites, trop vertes. Je peux tirer ? Elles sont trop petites. Amir lâche la fane. Pas d'orange. Pas cette fois. Le marché a des carottes. Le tuyau d'arrosage est froid sous le doigt. Il est froid ! On rentre. Amir retire le manteau. Il le raccroche au crochet. Le crochet fait un petit tic. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>éclat de cuillère</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,78 +1326,75 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_les_carottes_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une cuillère en bois sèche près de l'évier.
-narrateur|La soupe sent encore dans la cuisine.
-narrateur|La vitre a un peu de buée.
-narrateur|Dehors, le tuyau d'arrosage est enroulé.
-narrateur|Papa plie un sac de toile.
-papa|Amir, tu as vu la buée ?
+          <t>narrateur|La cuillère en bois tient dans un verre.
+narrateur|Elle sèche, un peu penchée, près de l'évier.
+narrateur|Un éclat de cuillère brille sur le bois.
+narrateur|Il est pâle, lisse, et il sent la soupe.
+narrateur|La casserole fume, trop claire.
+enfant-m|Il manque l'orange, papa.
+papa|Les carottes, Amir ?
+enfant-m|Oui, maintenant !
+narrateur|La buée dessine un trait tordu sur la vitre.
+narrateur|Dehors, le tuyau d'arrosage dort enroulé.
+narrateur|Papa plie le sac de toile, près du crochet.
+papa|Amir, tu as vu l'éclat ?
+enfant-m|Oui, il brille.
+narrateur|En ce moment, Amir veut les carottes.
+enfant-m|On y va, tout de suite !
+papa|D'abord le jardin.
+papa|Une carotte est peut-être prête.
+narrateur|Amir saisit le sac de toile.
+narrateur|Il court vers la porte, sans le manteau.
+enfant-m|Je sors, papa !
+narrateur|La porte s'ouvre.
+narrateur|L'air froid pique les poignets.
+narrateur|La sangle glisse, le sac tombe.
+enfant-m|Aïe !
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tes poignets sont froids ?
 enfant-m|Oui.
-enfant-m|On dirait un nuage.
-narrateur|En ce moment, Amir essuie un peu la buée.
-narrateur|Son manteau vert attend au crochet.
-papa|On va d'abord au jardin.
-papa|Le tuyau a peut-être de l'eau.
-papa|Avant de sortir, on prend le manteau.
-narrateur|Amir prend le manteau vert.
-narrateur|Il est un peu épais.
+enfant-m|Le sac est tombé.
+narrateur|Le manteau vert attend au crochet.
+narrateur|Ce manteau est un peu épais.
+narrateur|Le tissu gratte sous les doigts.
 narrateur|Amir glisse un bras, puis l'autre.
 papa|Tu es prêt ?
 enfant-m|Oui, papa.
-narrateur|Papa lace les chaussures d'Amir.
-narrateur|Ils vont au jardin.
-narrateur|L'air est frais.
+narrateur|Ils passent au jardin.
+narrateur|Une dalle est froide sous la semelle.
+enfant-m|Le sol pique.
+narrateur|Le coin du tuyau sent l'eau.
+narrateur|L'air sent l'herbe mouillée.
 narrateur|Amir touche une feuille lisse.
 enfant-m|Elle sent le jardin.
-papa|Oui.
-papa|Un peu l'herbe.
-papa|Un peu l'eau.
-narrateur|Le tuyau d'arrosage est froid.
-narrateur|Amir le touche du doigt.
+papa|Regarde les fanes.
+narrateur|Les fanes sont petites, trop vertes.
+enfant-m|Je peux tirer ?
+papa|Elles sont trop petites.
+narrateur|Amir lâche la fane.
+enfant-m|Pas d'orange.
+papa|Pas cette fois.
+papa|Le marché a des carottes.
+narrateur|Le tuyau d'arrosage est froid sous le doigt.
 enfant-m|Il est froid !
-papa|Oui.
-papa|C'est l'heure de rentrer.
-narrateur|Amir entre.
-narrateur|Il retire le manteau.
+papa|On rentre.
+narrateur|Amir retire le manteau.
 narrateur|Il le raccroche au crochet.
-narrateur|Le manteau vert est à sa place.
-narrateur|Plus tard, le sac de toile attend.
-papa|On va au marché, maintenant.
-papa|Pour les carottes de la soupe.
-narrateur|Amir se souvient.
-narrateur|Il va vers le crochet.
-narrateur|Le sac de toile cache le manteau.
-enfant-m|Je ne vois plus le manteau.
-papa|Le sac est devant.
-papa|Tu peux le déplacer ?
-narrateur|Amir pousse le sac tout doux.
-narrateur|Le manteau vert réapparaît.
-narrateur|Avant de sortir, il le prend.
-narrateur|Le même manteau vert.
-papa|Tu t'es souvenu tout seul.
-narrateur|Au marché, ça sent le pain.
-narrateur|Papa achète une botte de carottes.
-enfant-m|Elles sont orange.
-papa|Oui.
-papa|On les met dans le sac.
-narrateur|Puis ils rentrent.
-narrateur|Amir raccroche encore le manteau.
-narrateur|Le crochet fait le même petit bruit.
-enfant-m|Deux fois, papa.
-papa|Oui.
-papa|Deux fois.
-narrateur|Amir pose le sac de toile.
-narrateur|Les carottes font un petit bruit.
-papa|Tu as fini de poser le sac ?
-enfant-m|Oui, papa.</t>
+narrateur|Le crochet fait un petit tic.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>evier,porte</t>
+          <t>evier,casserole,porte</t>
         </is>
       </c>
     </row>
@@ -1429,12 +1426,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Amir ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Avant de &lt;emphasis level="moderate"&gt;sortir&lt;/emphasis&gt;, que prend Amir ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Avant de &lt;emphasis&gt;sortir&lt;/emphasis&gt;, que prend Violette ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Avant de &lt;emphasis&gt;sortir&lt;/emphasis&gt;, que prend Amir ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1497,7 +1494,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1505,10 +1502,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1523,11 +1520,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1538,23 +1535,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1563,23 +1560,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=avant_de_sortir_il_prend_le_manteau; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1611,17 +1608,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir a pris le manteau. Au jardin, puis au marché. Deux sorties. Le même manteau vert. En rentrant, il l'a raccroché. Tu t'es souvenu. Il est au crochet. Oui.</t>
+          <t>Amir a pris le manteau vert. Au jardin, les fanes étaient trop vertes. Le manteau est revenu au crochet. Le marché, maintenant. Pour les carottes de la soupe. Papa prend le sac de toile. Il le pose devant le crochet. Le sac cache le manteau vert. Je ne vois plus le manteau. On y va avec le sac ! Amir tire le sac, d'un coup. Le sac reste coincé contre le crochet. Ça ne veut pas. Ses épaules tombent. Tu regardes le crochet ? Amir serre le sac, puis le lâche. La buée revient sur la vitre. Elle cache un peu le crochet. Je sors avec le sac !</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir a pris le manteau. Au jardin, puis au marché. Deux sorties. Le même manteau vert. En rentrant, il l'a raccroché. Tu t'es souvenu. Il est au crochet. Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir a pris le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt; vert. Au jardin, les fanes étaient trop vertes. Le manteau est revenu au crochet. Le marché, maintenant. Pour les carottes de la soupe. Papa prend le sac de toile. Il le pose devant le crochet. Le sac cache le manteau vert. Je ne vois plus le manteau. On y va avec le sac ! Amir tire le sac, d'un coup. Le sac reste coincé contre le crochet. Ça ne veut pas. Ses épaules tombent. Tu regardes le crochet ? Amir serre le sac, puis le lâche. La buée revient sur la vitre. Elle cache un peu le crochet. Je sors avec le sac !&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Violette a pris le &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Au jardin, puis au marché. En rentrant, elle l'a raccroché. [pause]</t>
+          <t>Amir a pris le &lt;emphasis&gt;manteau&lt;/emphasis&gt; vert. Au jardin, les fanes étaient trop vertes. Le manteau est revenu au crochet. Le marché, maintenant. Pour les carottes de la soupe. Papa prend le sac de toile. Il le pose devant le crochet. Le sac cache le manteau vert. Je ne vois plus le manteau. On y va avec le sac ! Amir tire le sac, d'un coup. Le sac reste coincé contre le crochet. Ça ne veut pas. Ses épaules tombent. Tu regardes le crochet ? Amir serre le sac, puis le lâche. La buée revient sur la vitre. Elle cache un peu le crochet. Je sors avec le sac ! [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1668,7 +1665,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1676,10 +1673,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1706,7 +1703,7 @@
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
         <v>450</v>
@@ -1716,16 +1713,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1734,10 +1731,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1750,19 +1747,35 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=élan_impatient; intensite=1; destinataire=enfant; sous_texte=le_sac_cache_le_manteau; tempo=naturel; sourire=léger puis tendu; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir a pris le manteau.
-narrateur|Au jardin, puis au marché.
-narrateur|Deux sorties.
-narrateur|Le même manteau vert.
-narrateur|En rentrant, il l'a raccroché.
-papa|Tu t'es souvenu.
-enfant-m|Il est au crochet.
-papa|Oui.</t>
+          <t>narrateur|Amir a pris le manteau vert.
+narrateur|Au jardin, les fanes étaient trop vertes.
+narrateur|Le manteau est revenu au crochet.
+papa|Le marché, maintenant.
+papa|Pour les carottes de la soupe.
+narrateur|Papa prend le sac de toile.
+narrateur|Il le pose devant le crochet.
+narrateur|Le sac cache le manteau vert.
+enfant-m|Je ne vois plus le manteau.
+enfant-m|On y va avec le sac !
+narrateur|Amir tire le sac, d'un coup.
+narrateur|Le sac reste coincé contre le crochet.
+enfant-m|Ça ne veut pas.
+narrateur|Ses épaules tombent.
+papa|Tu regardes le crochet ?
+narrateur|Amir serre le sac, puis le lâche.
+narrateur|La buée revient sur la vitre.
+narrateur|Elle cache un peu le crochet.
+enfant-m|Je sors avec le sac !</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>sac,crochet</t>
         </is>
       </c>
     </row>
@@ -1789,17 +1802,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Amir pose les chaussures. Le manteau reste au crochet. Papa pose les carottes près de l'évier. Tu as fini de poser tes chaussures ? Oui, papa. La cuillère en bois est sèche. La buée a disparu de la vitre. On a les carottes pour la soupe. Le manteau aussi a travaillé. Oui. Le manteau aussi.</t>
+          <t>Amir refuse de foncer. Attends, je regarde. Personne ne dit le chemin. Amir écoute la cuisine. La casserole chuchote. Sur le verre, l'éclat de cuillère tremble. Il penche vers le crochet. C'est là ! Amir pousse le sac de côté. Le manteau vert réapparaît. Il glisse un bras, puis l'autre. Merci, Amir. On ouvre la porte ? Oui, avec le manteau. Au marché, ça sent le pain. L'étal orange est bas, près des caisses. Une caisse craque sous une botte. Tu vois les carottes ? Elles sont orange. Papa achète une botte de carottes. Ils les glissent dans le sac. Le sac de toile sent la terre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Amir pose les chaussures. Le manteau reste au crochet. Papa pose les carottes près de l'évier. Tu as fini de poser tes chaussures ? Oui, papa. La cuillère en bois est sèche. La buée a disparu de la vitre. On a les carottes pour la soupe. Le manteau aussi a travaillé. Oui. Le manteau aussi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir refuse de foncer. Attends, je regarde. Personne ne dit le chemin. Amir écoute la cuisine. La casserole chuchote. Sur le verre, l'&lt;emphasis level="moderate"&gt;éclat de cuillère&lt;/emphasis&gt; tremble. Il penche vers le crochet. C'est là ! Amir pousse le sac de côté. Le manteau vert réapparaît. Il glisse un bras, puis l'autre. Merci, Amir. On ouvre la porte ? Oui, avec le manteau. Au marché, ça sent le pain. L'étal orange est bas, près des caisses. Une caisse craque sous une botte. Tu vois les carottes ? Elles sont orange. Papa achète une botte de carottes. Ils les glissent dans le sac. Le sac de toile sent la terre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Violette pose les chaussures. Le &lt;emphasis&gt;manteau&lt;/emphasis&gt; reste au crochet. [pause]</t>
+          <t>Amir refuse de foncer. Attends, je regarde. Personne ne dit le chemin. Amir écoute la cuisine. La casserole chuchote. Sur le verre, l'&lt;emphasis&gt;éclat de cuillère&lt;/emphasis&gt; tremble. Il penche vers le crochet. C'est là ! Amir pousse le sac de côté. Le manteau vert réapparaît. Il glisse un bras, puis l'autre. Merci, Amir. On ouvre la porte ? Oui, avec le manteau. Au marché, ça sent le pain. L'étal orange est bas, près des caisses. Une caisse craque sous une botte. Tu vois les carottes ? Elles sont orange. Papa achète une botte de carottes. Ils les glissent dans le sac. Le sac de toile sent la terre. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1846,7 +1859,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1854,10 +1867,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1880,30 +1893,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>éclat de cuillère</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1912,10 +1925,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1926,20 +1939,40 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_l_éclat_montre_le_crochet; tempo=naturel; sourire=franc; respiration=relâchée</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose les chaussures.
-narrateur|Le manteau reste au crochet.
-narrateur|Papa pose les carottes près de l'évier.
-papa|Tu as fini de poser tes chaussures ?
-enfant-m|Oui, papa.
-narrateur|La cuillère en bois est sèche.
-narrateur|La buée a disparu de la vitre.
-papa|On a les carottes pour la soupe.
-enfant-m|Le manteau aussi a travaillé.
-papa|Oui.
-papa|Le manteau aussi.</t>
+          <t>narrateur|Amir refuse de foncer.
+enfant-m|Attends, je regarde.
+narrateur|Personne ne dit le chemin.
+narrateur|Amir écoute la cuisine.
+enfant-m|La casserole chuchote.
+narrateur|Sur le verre, l'éclat de cuillère tremble.
+narrateur|Il penche vers le crochet.
+enfant-m|C'est là !
+narrateur|Amir pousse le sac de côté.
+narrateur|Le manteau vert réapparaît.
+narrateur|Il glisse un bras, puis l'autre.
+papa|Merci, Amir.
+papa|On ouvre la porte ?
+enfant-m|Oui, avec le manteau.
+narrateur|Au marché, ça sent le pain.
+narrateur|L'étal orange est bas, près des caisses.
+narrateur|Une caisse craque sous une botte.
+papa|Tu vois les carottes ?
+enfant-m|Elles sont orange.
+narrateur|Papa achète une botte de carottes.
+narrateur|Ils les glissent dans le sac.
+narrateur|Le sac de toile sent la terre.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>marche,sac,caisse</t>
         </is>
       </c>
     </row>
@@ -1966,17 +1999,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai pris le manteau deux fois. Jardin, puis marché. Et tu l'as raccroché. Bravo, Amir. Les carottes attendent près de l'évier.</t>
+          <t>Amir pose les chaussures près de la porte. Le manteau vert reste au crochet. Papa pose les carottes près de l'évier. Tu as fini de poser tes chaussures ? Oui, papa. Papa coupe un rond orange. Le rond tombe dans la vapeur. La cuillère reprend sa place dans le verre. L'éclat a une trace. La soupe la prend. La buée a quitté la vitre. L'éclat de cuillère porte une trace orange.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai pris le manteau deux fois. Jardin, puis marché. Et tu l'as raccroché. Bravo, Amir. Les carottes attendent près de l'évier.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir pose les chaussures près de la porte. Le manteau vert reste au crochet. Papa pose les carottes près de l'évier. Tu as fini de poser tes chaussures ? Oui, papa. Papa coupe un rond orange. Le rond tombe dans la vapeur. La cuillère reprend sa place dans le verre. L'éclat a une trace. La soupe la prend. La buée a quitté la vitre. L'&lt;emphasis level="moderate"&gt;éclat de cuillère&lt;/emphasis&gt; porte une trace orange.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir pose les chaussures près de la porte. Le manteau vert reste au crochet. Papa pose les carottes près de l'évier. Tu as fini de poser tes chaussures ? Oui, papa. Papa coupe un rond orange. Le rond tombe dans la vapeur. La cuillère reprend sa place dans le verre. L'éclat a une trace. La soupe la prend. La buée a quitté la vitre. L'&lt;emphasis&gt;éclat de cuillère&lt;/emphasis&gt; porte une trace orange.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2023,15 +2056,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2043,12 +2076,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2057,17 +2090,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cuillère</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2076,11 +2113,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2089,28 +2126,44 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_éclat_porte_une_trace_orange; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai pris le manteau deux fois.
-enfant-m|Jardin, puis marché.
-papa|Et tu l'as raccroché.
-papa|Bravo, Amir.
-narrateur|Les carottes attendent près de l'évier.</t>
+          <t>narrateur|Amir pose les chaussures près de la porte.
+narrateur|Le manteau vert reste au crochet.
+narrateur|Papa pose les carottes près de l'évier.
+papa|Tu as fini de poser tes chaussures ?
+enfant-m|Oui, papa.
+narrateur|Papa coupe un rond orange.
+narrateur|Le rond tombe dans la vapeur.
+narrateur|La cuillère reprend sa place dans le verre.
+enfant-m|L'éclat a une trace.
+papa|La soupe la prend.
+narrateur|La buée a quitté la vitre.
+narrateur|L'éclat de cuillère porte une trace orange.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>casserole,evier</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2223,6 +2276,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>